<commit_message>
ADD: basic modification post reviews
</commit_message>
<xml_diff>
--- a/outreach_tracker.xlsx
+++ b/outreach_tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Contact form (insights4print.ceo/contact)</t>
+          <t>eddy.hagen@insights4print.ceo</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Sent via contact form</t>
+          <t>REPLIED - sent detailed color-stability answer, offered a call</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1817,11 +1817,19 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Needs manual submit (CAPTCHA)</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+          <t>Sent via contact form</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>Form at trade-show-advisor.com/trade-show-advisor-contact-form.html requires ticking I'm-not-a-robot - Manish to submit</t>
@@ -1866,7 +1874,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1913,11 +1921,19 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Filled - needs manual CAPTCHA + submit</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+          <t>Sent via contact form</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr">
         <is>
           <t>Form is filled in on an open Chrome tab; Manish just ticks I'm-not-a-robot and clicks Submit</t>
@@ -1971,32 +1987,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Classic Exhibits</t>
+          <t>American Image Displays</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>exhibitoradvocacy.com</t>
+          <t>insurancecanopy.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PR / Source relationship</t>
+          <t>Resource partnership / expert tip</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Joe Federbush (Founder)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>info@exhibitoradvocacy.com</t>
+          <t>info@insurancecanopy.com</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Supporting exhibitor-side transparency - from the print side</t>
+          <t>Same customers, different needs: vendor insurance + booth graphics</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2006,7 +2022,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2016,93 +2032,101 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Nonprofit exhibitor advocacy association; pitched as a printing-side source and asked about vendor alignment/listing</t>
+          <t>Insures market vendors/exhibitors (same customer base); site geo-blocked, email from search result</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Classic Exhibits</t>
+          <t>Vendor market outreach</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>scubefixtures.com</t>
+          <t>growingrootspartners.com (Craft + Mercantile night market, PA)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>N/A - competitor</t>
+          <t>Resource listing (vendor policy page)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Christy</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>christy@growingrootspartners.com</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>White 10x10 canopy tents for Craft + Mercantile vendors</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Skipped - competitor, not a partner</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Actually a portable display/fixture manufacturer competing in adjacent hardware space, not a partnership fit</t>
+          <t>Vendor policy explicitly requires a white 10x10 canopy tent - no supplier named</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Xibit Solutions</t>
+          <t>Vendor market outreach</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>elev8.la</t>
+          <t>tempefestivalofthearts.com (Dec 4-6 2026)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Backlink / co-marketing partnership</t>
+          <t>Resource listing (FAQ page)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Grant Morningstar (CEO)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>hello@elev8.la</t>
+          <t>events@downtowntempe.com</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Booth staffing + booth graphics - referral partnership?</t>
+          <t>White canopy tents + booth signage for Dec 4-6 Tempe artists</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>REPLIED - wants our service list</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2112,39 +2136,39 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Event staffing/brand ambassador agency (Las Vegas) - complementary, non-competing service for the same exhibitors</t>
+          <t>FAQ prefers white tents w/ 40lb weights per leg for ~350 accepted artists twice a year</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Impact XM</t>
+          <t>Vendor market outreach</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eventindustrynews.com</t>
+          <t>midwestcityok.org (Covered in Color)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PR / Source relationship</t>
+          <t>Resource listing (application page)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Adam Parry (Editor)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>editor@eventindustrynews.com</t>
+          <t>SpecialEvents@MidwestCityOK.org</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Printing/production-side source for event industry stories</t>
+          <t>Tent + booth signage resource for Covered in Color vendors</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2154,7 +2178,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2164,24 +2188,24 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>UK event industry trade news site; address came from a search result, not listed on-site - watch for bounce</t>
+          <t>Vendor application strongly recommends own tent, tables, signage - no supplier named</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Impact XM</t>
+          <t>Vendor market outreach</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>engine.com</t>
+          <t>hudsonvalleyopenmarket.com (2026 vendor info)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PR / Roundup inclusion</t>
+          <t>Resource listing (vendor info page)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2191,41 +2215,49 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>No form - support chat/phone only</t>
+          <t>hudsonvalleyopenmarket@gmail.com</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tent + weights + banner resource for Hudson Valley vendors</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Skipped - no contact form exists</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Sports event planning roundup; engine.com/contact-us</t>
+          <t>Vendor info requires 10x10 tent + 25lb weight per leg - specific setup, no supplier named</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Impact XM</t>
+          <t>Vendor market outreach</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>spotme.com</t>
+          <t>chiceventsdc.com (Royal Events Group, 16+ DC-area markets/yr)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Referral / resource partnership</t>
+          <t>Resource listing across event calendar</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2235,12 +2267,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>americas@spotme.com</t>
+          <t>ArtsandCrafts@Royal-EventsPlanning.com</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Partnership idea: SpotMe events + printed booth graphics</t>
+          <t>Tent + banner resource for your 16+ DC-area markets</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2250,7 +2282,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2260,39 +2292,39 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Enterprise event platform, 'best hybrid event management companies' roundup; spotme.com/contact-us</t>
+          <t>Runs National Harbor, Kentlands, Alexandria + other markets; vendors bring own tent, may hang booth signage</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Impact XM</t>
+          <t>E-Z UP</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>bizzabo.com</t>
+          <t>artsgoggle.org (Fort Worth art festival)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PR / Blog feature</t>
+          <t>Resource listing (artist info page)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Blog team</t>
+          <t>Natalie Atkinson (Events + Projects Manager)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>blog@bizzabo.com</t>
+          <t>natalie@nearsouthsidefw.org</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Feature idea: the printed side of corporate event themes</t>
+          <t>Booth tent + banner resource for ArtsGoggle artists</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2302,7 +2334,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2312,49 +2344,49 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Event platform, corporate event themes blog; bizzabo.com/contact-us</t>
+          <t>1,000+ artist booths, Oct 24 2026; artist-info page currently recommends E-Z UP tents</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Impact XM</t>
+          <t>Classic Exhibits</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>avenuez.com</t>
+          <t>exhibitoradvocacy.com</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PR / Roundup inclusion</t>
+          <t>PR / Source relationship</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Joe Federbush (Founder)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Contact form (avenuez.com/contact-us)</t>
+          <t>info@exhibitoradvocacy.com</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Contact form: referral partnership / guide mention</t>
+          <t>Supporting exhibitor-side transparency - from the print side</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Sent via contact form</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2364,34 +2396,34 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Beauty/wellness event PR agency, roundup lists Avenue Z itself first; avenuez.com/contact-us</t>
+          <t>Nonprofit exhibitor advocacy association; pitched as a printing-side source and asked about vendor alignment/listing</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3D Exhibits / Expo Marketing</t>
+          <t>Classic Exhibits</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>wearesparks.com</t>
+          <t>scubefixtures.com</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PR / Source relationship</t>
+          <t>N/A - competitor</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kristin Castelli (SVP Strategic Growth)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Lead form only - no message field</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2401,12 +2433,360 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Skipped - form cannot carry a message</t>
+          <t>Skipped - competitor, not a partner</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
+        <is>
+          <t>Actually a portable display/fixture manufacturer competing in adjacent hardware space, not a partnership fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Xibit Solutions</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>elev8.la</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Backlink / co-marketing partnership</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Grant Morningstar (CEO)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>hello@elev8.la</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Booth staffing + booth graphics - referral partnership?</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Replied - service list sent, call proposed</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Event staffing/brand ambassador agency (Las Vegas) - complementary, non-competing service for the same exhibitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Impact XM</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>eventindustrynews.com</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PR / Source relationship</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Adam Parry (Editor)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>editor@eventindustrynews.com</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Printing/production-side source for event industry stories</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>UK event industry trade news site; address came from a search result, not listed on-site - watch for bounce</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Impact XM</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>engine.com</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PR / Roundup inclusion</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>No form - support chat/phone only</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Skipped - no contact form exists</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Sports event planning roundup; engine.com/contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Impact XM</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>spotme.com</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Referral / resource partnership</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>americas@spotme.com</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Partnership idea: SpotMe events + printed booth graphics</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Enterprise event platform, 'best hybrid event management companies' roundup; spotme.com/contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Impact XM</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>bizzabo.com</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PR / Blog feature</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Blog team</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>blog@bizzabo.com</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Feature idea: the printed side of corporate event themes</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Event platform, corporate event themes blog; bizzabo.com/contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Impact XM</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>avenuez.com</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PR / Roundup inclusion</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Contact form (avenuez.com/contact-us)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Contact form: referral partnership / guide mention</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Sent via contact form</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>marketing@apextradeshow.com</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Beauty/wellness event PR agency, roundup lists Avenue Z itself first; avenuez.com/contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>3D Exhibits / Expo Marketing</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>wearesparks.com</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PR / Source relationship</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Kristin Castelli (SVP Strategic Growth)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Lead form only - no message field</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Skipped - form cannot carry a message</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
         <is>
           <t>Global healthcare/experiential brand agency, appeared as referrer for both Expo Marketing and 3D Exhibits; wearesparks.com/contact/</t>
         </is>
@@ -2423,7 +2803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2838,23 +3218,148 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>showdowndisplays.com</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>57</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>116K</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1.2K</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Wholesale tent/flag/banner supplier sold through promo distributors - backlinks are resellers' vendor-link pages (a wholesale/reseller channel, not editorial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>vispronet.com</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16K</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1.6K</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Online tent/banner printer - earns links from its own how-to guides (pride flags, sublimation, hanging banners) being cited; few outreach targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>241K</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1.6K</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Trade show exhibit company - strong content/expert-quote links (tip roundups, small-biz blogs, AI Journal, Insurance Canopy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tradeshowdisplaypros.com</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5.1K</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>983</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Low authority; links are mostly paid guest posts on general blogs and competitor pages - nothing new to pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ezup.com</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>52</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2.8K</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Canopy tent brand - top links come from teacher/military/first-responder discount lists (VA News DR91, Parade DR85) and festival vendor-info pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>ges.com</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B22" t="n">
         <v>71</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>59K</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>4.7K</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Global exhibition services giant - referrers mostly venues, associations, and exhibitor service portals (not editorial content); no new usable contacts found</t>
         </is>
@@ -2871,7 +3376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3869,12 +4374,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Needs manual submit</t>
+          <t>Sent via contact form</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Form has an I'm-not-a-robot CAPTCHA - Manish must submit</t>
+          <t>Confirmed - publisher Jules Sowder</t>
         </is>
       </c>
     </row>
@@ -7042,12 +7547,642 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Needs manual submit</t>
+          <t>Sent via contact form</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Form filled; CAPTCHA checkbox needs Manish</t>
+          <t>Confirmed by Joe Lynch auto-thanks</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>showdowndisplays.com</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>keystonead / majormktg / batcity / logoexpressions / joshowpromos / psprinting / prg.ca / doolittlesprintserve / bflprinting / signproiowa / prodesigns365</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>2-36</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Promo distributors' supplier pages - requires a wholesale program</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>showdowndisplays.com</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>flagpro / maximumpro / walloffameproducts / americanoutfitters / nifda.net</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>10-29</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Resellers / flag dealer association</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>showdowndisplays.com</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>members.asicentral.com / grokipedia / chemicalsamerica / printleaf</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>37-79</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>ASI members-only / aggregators / resellers</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>vispronet.com</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>vispronet.de / .at / .fr / .eu</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>3-34</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Own international sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>vispronet.com</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>wikipedia / wikihow / hunker / gemstonelights / matadormeggings / interestingfacts / artglasssupplies / lakeshorefablab</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>7-97</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Citations of Vispronet's blog guides - content, not outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>vispronet.com</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>impact-nw.com</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>23</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Competitor - skipped</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Print shop</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>vispronet.com</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>simplycodes / saver / bbb</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>11-93</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Coupons / profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>vispronet.com</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>adamchristing.com / ampddesigns / creekroadrentals / heartlandanimalshelter</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>6-34</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Low relevance</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>insurancecanopy.com</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>70</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Sent (see tracker)</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>info@insurancecanopy.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>tablelegsonline.com</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>31</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Expert-tip roundup but phone-only contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>zachwaldman.com</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>31</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Contact form / no public email</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Trade show magician - booking form only</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>badgermapping.com</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>68</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Contact form / no public email</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Sales software blog - contact form only</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>experiumagency.com</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>8</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Competitor - skipped</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>UK exhibition stand company</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>tradeshowlabs.com</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>57</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Sent (see tracker)</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Already contacted</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>wavecnct / noahpinion / voices / ahaslides / dunelandmedia / marketing-resultats / topleftdesign / carolroth / aijourn / lookwhatmomfound / olympiaartleague / grokipedia</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>12-78</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Citations of American Image's content, off-topic or low fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>american-image.com</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>exhibit-design-search / myshopify</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>56-95</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>American Image's own properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>tradeshowdisplaypros.com</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>anyvoo / vocal.media / 4mark / techbii / computertechreviews / teamgate / mikegingerich / logingit / metalplastikcelik / 1ptdesign</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>0-82</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Paid guest posts / off-topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>tradeshowdisplaypros.com</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>arrowheadsigncompany / displaystandsmarket / iconicdisplays / amitoje / vdshowcase</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>1-33</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Competitor - skipped</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Sign/display companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>tradeshowdisplaypros.com</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>print.wiki / sitelike / accio / alldatabases / yolasite</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>15-84</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Glossary / aggregators / own mirror</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>ezup.com</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>news.va.gov / parade / collegetransitions / teacherscan / dontpayfull</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>12-91</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Discount lists - need a teacher/military/first-responder discount program (Manish's decision)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>ezup.com</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>artsgoggle.org</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>35</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Sent (see tracker)</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>natalie@nearsouthsidefw.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>ezup.com</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>ezup.nl / .ca / .eu / .fr / .de / adidas-team</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>19-55</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>E-Z UP's own sites / co-brand store</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>ezup.com</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>westshade.com</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>17</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Competitor - skipped</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Canopy competitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>ezup.com</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>swiftotter / hawksem / boast.io / cmc.com / pnw4wda / drinkluckyduck / simplycodes</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>0-75</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Not actionable</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Agency case studies, coupons, off-topic</t>
         </is>
       </c>
     </row>

</xml_diff>